<commit_message>
chore: actualizar plantillas Excel de horarios por grupo
</commit_message>
<xml_diff>
--- a/Template_Horarios_Grupos_Matutino_5.xlsx
+++ b/Template_Horarios_Grupos_Matutino_5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\source\repos\CBTis73\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AFBA575F-B9F1-4AED-890D-C269597A0FE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B4604A9-FC43-4B9E-9BAE-E3B067C3E97D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="23596" windowHeight="15076" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -450,13 +450,31 @@
     <xf numFmtId="0" fontId="11" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="20" fontId="13" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -465,6 +483,48 @@
     <xf numFmtId="20" fontId="13" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="20" fontId="13" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="13" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="11" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="11" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="16" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="16" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="16" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="16" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="20" fontId="10" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -474,92 +534,32 @@
     <xf numFmtId="20" fontId="10" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="13" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="13" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="16" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="16" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="11" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="11" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="16" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="16" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1152,22 +1152,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:15" ht="25.5" x14ac:dyDescent="0.75">
-      <c r="D1" s="47" t="s">
+      <c r="D1" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="47"/>
-      <c r="F1" s="47"/>
-      <c r="G1" s="47"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
       <c r="H1" s="1"/>
       <c r="I1" s="2"/>
     </row>
     <row r="2" spans="2:15" ht="18" x14ac:dyDescent="0.55000000000000004">
-      <c r="D2" s="48" t="s">
+      <c r="D2" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="48"/>
-      <c r="F2" s="48"/>
-      <c r="G2" s="48"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
       <c r="H2" s="4"/>
       <c r="I2" s="5"/>
       <c r="J2">
@@ -1188,12 +1188,12 @@
     </row>
     <row r="4" spans="2:15" ht="20.65" x14ac:dyDescent="0.6">
       <c r="C4" s="6"/>
-      <c r="D4" s="49"/>
-      <c r="E4" s="49"/>
-      <c r="F4" s="50" t="s">
+      <c r="D4" s="25"/>
+      <c r="E4" s="25"/>
+      <c r="F4" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="G4" s="50"/>
+      <c r="G4" s="29"/>
       <c r="H4" s="6"/>
       <c r="I4" s="5"/>
       <c r="J4">
@@ -1216,15 +1216,15 @@
       <c r="B6" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="51" t="s">
+      <c r="C6" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="52"/>
-      <c r="E6" s="53" t="s">
+      <c r="D6" s="27"/>
+      <c r="E6" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="F6" s="53"/>
-      <c r="G6" s="53"/>
+      <c r="F6" s="28"/>
+      <c r="G6" s="28"/>
       <c r="H6" s="8"/>
       <c r="I6" s="5"/>
       <c r="J6">
@@ -1281,14 +1281,14 @@
       <c r="O8"/>
     </row>
     <row r="9" spans="2:15" s="13" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B9" s="54" t="s">
+      <c r="B9" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="43"/>
-      <c r="D9" s="43"/>
-      <c r="E9" s="43"/>
-      <c r="F9" s="43"/>
-      <c r="G9" s="43"/>
+      <c r="C9" s="34"/>
+      <c r="D9" s="34"/>
+      <c r="E9" s="34"/>
+      <c r="F9" s="34"/>
+      <c r="G9" s="34"/>
       <c r="H9" s="12"/>
       <c r="I9" s="5"/>
       <c r="J9">
@@ -1303,12 +1303,12 @@
       <c r="O9"/>
     </row>
     <row r="10" spans="2:15" s="13" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B10" s="55"/>
-      <c r="C10" s="44"/>
-      <c r="D10" s="44"/>
-      <c r="E10" s="44"/>
-      <c r="F10" s="44"/>
-      <c r="G10" s="44"/>
+      <c r="B10" s="37"/>
+      <c r="C10" s="35"/>
+      <c r="D10" s="35"/>
+      <c r="E10" s="35"/>
+      <c r="F10" s="35"/>
+      <c r="G10" s="35"/>
       <c r="H10" s="12"/>
       <c r="I10" s="5"/>
       <c r="J10">
@@ -1323,14 +1323,14 @@
       <c r="O10"/>
     </row>
     <row r="11" spans="2:15" s="13" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B11" s="56" t="s">
+      <c r="B11" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="43"/>
-      <c r="D11" s="43"/>
-      <c r="E11" s="43"/>
-      <c r="F11" s="43"/>
-      <c r="G11" s="43"/>
+      <c r="C11" s="34"/>
+      <c r="D11" s="34"/>
+      <c r="E11" s="34"/>
+      <c r="F11" s="34"/>
+      <c r="G11" s="34"/>
       <c r="H11" s="12"/>
       <c r="I11" s="5"/>
       <c r="J11">
@@ -1345,12 +1345,12 @@
       <c r="O11"/>
     </row>
     <row r="12" spans="2:15" s="13" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B12" s="57"/>
-      <c r="C12" s="44"/>
-      <c r="D12" s="44"/>
-      <c r="E12" s="44"/>
-      <c r="F12" s="44"/>
-      <c r="G12" s="44"/>
+      <c r="B12" s="31"/>
+      <c r="C12" s="35"/>
+      <c r="D12" s="35"/>
+      <c r="E12" s="35"/>
+      <c r="F12" s="35"/>
+      <c r="G12" s="35"/>
       <c r="H12" s="12"/>
       <c r="I12" s="5"/>
       <c r="J12">
@@ -1365,14 +1365,14 @@
       <c r="O12"/>
     </row>
     <row r="13" spans="2:15" s="13" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B13" s="54" t="s">
+      <c r="B13" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="43"/>
-      <c r="D13" s="43"/>
-      <c r="E13" s="43"/>
-      <c r="F13" s="43"/>
-      <c r="G13" s="45"/>
+      <c r="C13" s="34"/>
+      <c r="D13" s="34"/>
+      <c r="E13" s="34"/>
+      <c r="F13" s="34"/>
+      <c r="G13" s="38"/>
       <c r="H13" s="12"/>
       <c r="I13" s="5"/>
       <c r="J13">
@@ -1387,12 +1387,12 @@
       <c r="O13"/>
     </row>
     <row r="14" spans="2:15" s="13" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B14" s="55"/>
-      <c r="C14" s="44"/>
-      <c r="D14" s="44"/>
-      <c r="E14" s="44"/>
-      <c r="F14" s="44"/>
-      <c r="G14" s="46"/>
+      <c r="B14" s="37"/>
+      <c r="C14" s="35"/>
+      <c r="D14" s="35"/>
+      <c r="E14" s="35"/>
+      <c r="F14" s="35"/>
+      <c r="G14" s="39"/>
       <c r="H14" s="12"/>
       <c r="I14" s="5"/>
       <c r="J14">
@@ -1407,14 +1407,14 @@
       <c r="O14"/>
     </row>
     <row r="15" spans="2:15" s="13" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B15" s="56" t="s">
+      <c r="B15" s="30" t="s">
         <v>41</v>
       </c>
-      <c r="C15" s="26"/>
-      <c r="D15" s="26"/>
-      <c r="E15" s="26"/>
-      <c r="F15" s="26"/>
-      <c r="G15" s="26"/>
+      <c r="C15" s="32"/>
+      <c r="D15" s="32"/>
+      <c r="E15" s="32"/>
+      <c r="F15" s="32"/>
+      <c r="G15" s="32"/>
       <c r="H15" s="12"/>
       <c r="I15" s="5"/>
       <c r="J15">
@@ -1429,12 +1429,12 @@
       <c r="O15"/>
     </row>
     <row r="16" spans="2:15" s="13" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B16" s="57"/>
-      <c r="C16" s="27"/>
-      <c r="D16" s="27"/>
-      <c r="E16" s="27"/>
-      <c r="F16" s="27"/>
-      <c r="G16" s="27"/>
+      <c r="B16" s="31"/>
+      <c r="C16" s="33"/>
+      <c r="D16" s="33"/>
+      <c r="E16" s="33"/>
+      <c r="F16" s="33"/>
+      <c r="G16" s="33"/>
       <c r="H16" s="12"/>
       <c r="I16" s="5"/>
       <c r="J16">
@@ -1452,13 +1452,13 @@
       <c r="B17" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="C17" s="28" t="s">
+      <c r="C17" s="48" t="s">
         <v>43</v>
       </c>
-      <c r="D17" s="29"/>
-      <c r="E17" s="29"/>
-      <c r="F17" s="29"/>
-      <c r="G17" s="30"/>
+      <c r="D17" s="49"/>
+      <c r="E17" s="49"/>
+      <c r="F17" s="49"/>
+      <c r="G17" s="50"/>
       <c r="H17" s="12"/>
       <c r="I17" s="5"/>
       <c r="J17">
@@ -1473,14 +1473,14 @@
       <c r="O17"/>
     </row>
     <row r="18" spans="2:15" s="13" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B18" s="56" t="s">
+      <c r="B18" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="C18" s="43"/>
-      <c r="D18" s="26"/>
-      <c r="E18" s="43"/>
-      <c r="F18" s="58"/>
-      <c r="G18" s="26"/>
+      <c r="C18" s="34"/>
+      <c r="D18" s="32"/>
+      <c r="E18" s="34"/>
+      <c r="F18" s="40"/>
+      <c r="G18" s="32"/>
       <c r="H18" s="12"/>
       <c r="I18" s="5"/>
       <c r="J18">
@@ -1495,12 +1495,12 @@
       <c r="O18"/>
     </row>
     <row r="19" spans="2:15" s="13" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B19" s="57"/>
-      <c r="C19" s="44"/>
-      <c r="D19" s="27"/>
-      <c r="E19" s="44"/>
-      <c r="F19" s="59"/>
-      <c r="G19" s="27"/>
+      <c r="B19" s="31"/>
+      <c r="C19" s="35"/>
+      <c r="D19" s="33"/>
+      <c r="E19" s="35"/>
+      <c r="F19" s="41"/>
+      <c r="G19" s="33"/>
       <c r="H19" s="12"/>
       <c r="I19" s="5"/>
       <c r="J19">
@@ -1515,14 +1515,14 @@
       <c r="O19"/>
     </row>
     <row r="20" spans="2:15" s="13" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B20" s="56" t="s">
+      <c r="B20" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="C20" s="58"/>
-      <c r="D20" s="26"/>
-      <c r="E20" s="26"/>
-      <c r="F20" s="26"/>
-      <c r="G20" s="26"/>
+      <c r="C20" s="40"/>
+      <c r="D20" s="32"/>
+      <c r="E20" s="32"/>
+      <c r="F20" s="32"/>
+      <c r="G20" s="32"/>
       <c r="H20" s="12"/>
       <c r="I20" s="5"/>
       <c r="J20">
@@ -1537,12 +1537,12 @@
       <c r="O20"/>
     </row>
     <row r="21" spans="2:15" s="13" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B21" s="57"/>
-      <c r="C21" s="59"/>
-      <c r="D21" s="27"/>
-      <c r="E21" s="27"/>
-      <c r="F21" s="27"/>
-      <c r="G21" s="27"/>
+      <c r="B21" s="31"/>
+      <c r="C21" s="41"/>
+      <c r="D21" s="33"/>
+      <c r="E21" s="33"/>
+      <c r="F21" s="33"/>
+      <c r="G21" s="33"/>
       <c r="H21" s="12"/>
       <c r="I21" s="5"/>
       <c r="J21">
@@ -1557,14 +1557,14 @@
       <c r="O21"/>
     </row>
     <row r="22" spans="2:15" s="13" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B22" s="56" t="s">
+      <c r="B22" s="30" t="s">
         <v>13</v>
       </c>
-      <c r="C22" s="26"/>
-      <c r="D22" s="26"/>
-      <c r="E22" s="58"/>
-      <c r="F22" s="58"/>
-      <c r="G22" s="26"/>
+      <c r="C22" s="32"/>
+      <c r="D22" s="32"/>
+      <c r="E22" s="40"/>
+      <c r="F22" s="40"/>
+      <c r="G22" s="32"/>
       <c r="H22" s="12"/>
       <c r="I22" s="5"/>
       <c r="J22">
@@ -1579,12 +1579,12 @@
       <c r="O22"/>
     </row>
     <row r="23" spans="2:15" s="13" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B23" s="57"/>
-      <c r="C23" s="27"/>
-      <c r="D23" s="27"/>
-      <c r="E23" s="59"/>
-      <c r="F23" s="59"/>
-      <c r="G23" s="27"/>
+      <c r="B23" s="31"/>
+      <c r="C23" s="33"/>
+      <c r="D23" s="33"/>
+      <c r="E23" s="41"/>
+      <c r="F23" s="41"/>
+      <c r="G23" s="33"/>
       <c r="H23" s="12"/>
       <c r="I23" s="5"/>
       <c r="J23">
@@ -1599,14 +1599,14 @@
       <c r="O23"/>
     </row>
     <row r="24" spans="2:15" s="13" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B24" s="56" t="s">
+      <c r="B24" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="C24" s="26"/>
-      <c r="D24" s="26"/>
-      <c r="E24" s="26"/>
-      <c r="F24" s="58"/>
-      <c r="G24" s="43"/>
+      <c r="C24" s="32"/>
+      <c r="D24" s="32"/>
+      <c r="E24" s="32"/>
+      <c r="F24" s="40"/>
+      <c r="G24" s="34"/>
       <c r="H24" s="12"/>
       <c r="I24" s="5"/>
       <c r="J24">
@@ -1621,12 +1621,12 @@
       <c r="O24"/>
     </row>
     <row r="25" spans="2:15" s="13" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B25" s="57"/>
-      <c r="C25" s="27"/>
-      <c r="D25" s="27"/>
-      <c r="E25" s="27"/>
-      <c r="F25" s="59"/>
-      <c r="G25" s="44"/>
+      <c r="B25" s="31"/>
+      <c r="C25" s="33"/>
+      <c r="D25" s="33"/>
+      <c r="E25" s="33"/>
+      <c r="F25" s="41"/>
+      <c r="G25" s="35"/>
       <c r="H25" s="12"/>
       <c r="I25" s="5"/>
       <c r="J25">
@@ -1661,12 +1661,12 @@
       <c r="C27" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="D27" s="37" t="s">
+      <c r="D27" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="E27" s="38"/>
-      <c r="F27" s="38"/>
-      <c r="G27" s="39"/>
+      <c r="E27" s="45"/>
+      <c r="F27" s="45"/>
+      <c r="G27" s="46"/>
       <c r="H27" s="12"/>
       <c r="I27" s="5"/>
       <c r="J27">
@@ -1687,10 +1687,10 @@
       <c r="C28" s="15">
         <v>5</v>
       </c>
-      <c r="D28" s="34"/>
-      <c r="E28" s="35"/>
-      <c r="F28" s="35"/>
-      <c r="G28" s="36"/>
+      <c r="D28" s="51"/>
+      <c r="E28" s="52"/>
+      <c r="F28" s="52"/>
+      <c r="G28" s="53"/>
       <c r="H28" s="12"/>
       <c r="I28" s="5"/>
       <c r="J28">
@@ -1711,10 +1711,10 @@
       <c r="C29" s="15">
         <v>5</v>
       </c>
-      <c r="D29" s="34"/>
-      <c r="E29" s="35"/>
-      <c r="F29" s="35"/>
-      <c r="G29" s="36"/>
+      <c r="D29" s="51"/>
+      <c r="E29" s="52"/>
+      <c r="F29" s="52"/>
+      <c r="G29" s="53"/>
       <c r="H29" s="12"/>
       <c r="I29" s="5"/>
       <c r="J29">
@@ -1735,10 +1735,10 @@
       <c r="C30" s="15">
         <v>4</v>
       </c>
-      <c r="D30" s="40"/>
-      <c r="E30" s="41"/>
-      <c r="F30" s="41"/>
-      <c r="G30" s="42"/>
+      <c r="D30" s="54"/>
+      <c r="E30" s="55"/>
+      <c r="F30" s="55"/>
+      <c r="G30" s="56"/>
       <c r="H30" s="12"/>
       <c r="I30" s="5"/>
       <c r="J30">
@@ -1759,10 +1759,10 @@
       <c r="C31" s="15">
         <v>3</v>
       </c>
-      <c r="D31" s="40"/>
-      <c r="E31" s="41"/>
-      <c r="F31" s="41"/>
-      <c r="G31" s="42"/>
+      <c r="D31" s="54"/>
+      <c r="E31" s="55"/>
+      <c r="F31" s="55"/>
+      <c r="G31" s="56"/>
       <c r="H31" s="12"/>
       <c r="I31" s="5"/>
       <c r="J31">
@@ -1779,10 +1779,10 @@
       <c r="C32" s="15">
         <v>1</v>
       </c>
-      <c r="D32" s="34"/>
-      <c r="E32" s="35"/>
-      <c r="F32" s="35"/>
-      <c r="G32" s="36"/>
+      <c r="D32" s="51"/>
+      <c r="E32" s="52"/>
+      <c r="F32" s="52"/>
+      <c r="G32" s="53"/>
       <c r="H32" s="12"/>
       <c r="I32" s="5"/>
       <c r="J32">
@@ -1799,10 +1799,10 @@
       <c r="C33" s="15">
         <v>3</v>
       </c>
-      <c r="D33" s="40"/>
-      <c r="E33" s="41"/>
-      <c r="F33" s="41"/>
-      <c r="G33" s="42"/>
+      <c r="D33" s="54"/>
+      <c r="E33" s="55"/>
+      <c r="F33" s="55"/>
+      <c r="G33" s="56"/>
       <c r="H33" s="12"/>
       <c r="I33" s="5"/>
       <c r="J33">
@@ -1819,10 +1819,10 @@
       <c r="C34" s="15">
         <v>7</v>
       </c>
-      <c r="D34" s="34"/>
-      <c r="E34" s="35"/>
-      <c r="F34" s="35"/>
-      <c r="G34" s="36"/>
+      <c r="D34" s="51"/>
+      <c r="E34" s="52"/>
+      <c r="F34" s="52"/>
+      <c r="G34" s="53"/>
       <c r="H34" s="12"/>
       <c r="I34" s="5"/>
       <c r="J34">
@@ -1839,10 +1839,10 @@
       <c r="C35" s="15">
         <v>5</v>
       </c>
-      <c r="D35" s="34"/>
-      <c r="E35" s="35"/>
-      <c r="F35" s="35"/>
-      <c r="G35" s="36"/>
+      <c r="D35" s="51"/>
+      <c r="E35" s="52"/>
+      <c r="F35" s="52"/>
+      <c r="G35" s="53"/>
       <c r="H35" s="12"/>
       <c r="I35" s="5"/>
     </row>
@@ -1853,10 +1853,10 @@
       <c r="C36" s="15">
         <v>1</v>
       </c>
-      <c r="D36" s="40"/>
-      <c r="E36" s="41"/>
-      <c r="F36" s="41"/>
-      <c r="G36" s="42"/>
+      <c r="D36" s="54"/>
+      <c r="E36" s="55"/>
+      <c r="F36" s="55"/>
+      <c r="G36" s="56"/>
       <c r="H36" s="12"/>
       <c r="I36" s="5"/>
       <c r="J36">
@@ -1886,13 +1886,13 @@
       <c r="B38" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="C38" s="37" t="s">
+      <c r="C38" s="44" t="s">
         <v>19</v>
       </c>
-      <c r="D38" s="38"/>
-      <c r="E38" s="38"/>
-      <c r="F38" s="38"/>
-      <c r="G38" s="39"/>
+      <c r="D38" s="45"/>
+      <c r="E38" s="45"/>
+      <c r="F38" s="45"/>
+      <c r="G38" s="46"/>
       <c r="I38" s="5"/>
       <c r="J38">
         <v>39</v>
@@ -1903,20 +1903,20 @@
     </row>
     <row r="39" spans="2:12" ht="18" x14ac:dyDescent="0.45">
       <c r="B39" s="15"/>
-      <c r="C39" s="34"/>
-      <c r="D39" s="35"/>
-      <c r="E39" s="35"/>
-      <c r="F39" s="35"/>
-      <c r="G39" s="36"/>
+      <c r="C39" s="51"/>
+      <c r="D39" s="52"/>
+      <c r="E39" s="52"/>
+      <c r="F39" s="52"/>
+      <c r="G39" s="53"/>
       <c r="I39" s="5"/>
     </row>
     <row r="40" spans="2:12" ht="18" x14ac:dyDescent="0.45">
       <c r="B40" s="15"/>
-      <c r="C40" s="34"/>
-      <c r="D40" s="35"/>
-      <c r="E40" s="35"/>
-      <c r="F40" s="35"/>
-      <c r="G40" s="36"/>
+      <c r="C40" s="51"/>
+      <c r="D40" s="52"/>
+      <c r="E40" s="52"/>
+      <c r="F40" s="52"/>
+      <c r="G40" s="53"/>
       <c r="I40" s="5"/>
       <c r="J40">
         <v>40</v>
@@ -1927,11 +1927,11 @@
     </row>
     <row r="41" spans="2:12" ht="18" x14ac:dyDescent="0.45">
       <c r="B41" s="15"/>
-      <c r="C41" s="23"/>
-      <c r="D41" s="24"/>
-      <c r="E41" s="24"/>
-      <c r="F41" s="24"/>
-      <c r="G41" s="25"/>
+      <c r="C41" s="57"/>
+      <c r="D41" s="58"/>
+      <c r="E41" s="58"/>
+      <c r="F41" s="58"/>
+      <c r="G41" s="59"/>
       <c r="I41" s="5"/>
       <c r="J41">
         <v>41</v>
@@ -1942,11 +1942,11 @@
     </row>
     <row r="42" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B42" s="15"/>
-      <c r="C42" s="23"/>
-      <c r="D42" s="24"/>
-      <c r="E42" s="24"/>
-      <c r="F42" s="24"/>
-      <c r="G42" s="25"/>
+      <c r="C42" s="57"/>
+      <c r="D42" s="58"/>
+      <c r="E42" s="58"/>
+      <c r="F42" s="58"/>
+      <c r="G42" s="59"/>
       <c r="J42">
         <v>42</v>
       </c>
@@ -1956,11 +1956,11 @@
     </row>
     <row r="43" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B43" s="15"/>
-      <c r="C43" s="23"/>
-      <c r="D43" s="24"/>
-      <c r="E43" s="24"/>
-      <c r="F43" s="24"/>
-      <c r="G43" s="25"/>
+      <c r="C43" s="57"/>
+      <c r="D43" s="58"/>
+      <c r="E43" s="58"/>
+      <c r="F43" s="58"/>
+      <c r="G43" s="59"/>
       <c r="J43">
         <v>43</v>
       </c>
@@ -1970,11 +1970,11 @@
     </row>
     <row r="44" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B44" s="15"/>
-      <c r="C44" s="23"/>
-      <c r="D44" s="24"/>
-      <c r="E44" s="24"/>
-      <c r="F44" s="24"/>
-      <c r="G44" s="25"/>
+      <c r="C44" s="57"/>
+      <c r="D44" s="58"/>
+      <c r="E44" s="58"/>
+      <c r="F44" s="58"/>
+      <c r="G44" s="59"/>
       <c r="J44">
         <v>44</v>
       </c>
@@ -1984,11 +1984,11 @@
     </row>
     <row r="45" spans="2:12" ht="15.4" x14ac:dyDescent="0.45">
       <c r="B45" s="15"/>
-      <c r="C45" s="23"/>
-      <c r="D45" s="24"/>
-      <c r="E45" s="24"/>
-      <c r="F45" s="24"/>
-      <c r="G45" s="25"/>
+      <c r="C45" s="57"/>
+      <c r="D45" s="58"/>
+      <c r="E45" s="58"/>
+      <c r="F45" s="58"/>
+      <c r="G45" s="59"/>
       <c r="H45" s="9"/>
       <c r="J45">
         <v>45</v>
@@ -1999,11 +1999,11 @@
     </row>
     <row r="46" spans="2:12" ht="15.4" x14ac:dyDescent="0.45">
       <c r="B46" s="15"/>
-      <c r="C46" s="23"/>
-      <c r="D46" s="24"/>
-      <c r="E46" s="24"/>
-      <c r="F46" s="24"/>
-      <c r="G46" s="25"/>
+      <c r="C46" s="57"/>
+      <c r="D46" s="58"/>
+      <c r="E46" s="58"/>
+      <c r="F46" s="58"/>
+      <c r="G46" s="59"/>
       <c r="H46" s="9"/>
       <c r="J46">
         <v>46</v>
@@ -2014,11 +2014,11 @@
     </row>
     <row r="47" spans="2:12" ht="15.4" x14ac:dyDescent="0.45">
       <c r="B47" s="15"/>
-      <c r="C47" s="34"/>
-      <c r="D47" s="35"/>
-      <c r="E47" s="35"/>
-      <c r="F47" s="35"/>
-      <c r="G47" s="36"/>
+      <c r="C47" s="51"/>
+      <c r="D47" s="52"/>
+      <c r="E47" s="52"/>
+      <c r="F47" s="52"/>
+      <c r="G47" s="53"/>
       <c r="H47" s="9"/>
       <c r="J47">
         <v>47</v>
@@ -2057,16 +2057,16 @@
       </c>
     </row>
     <row r="50" spans="2:12" x14ac:dyDescent="0.45">
-      <c r="B50" s="33" t="s">
+      <c r="B50" s="47" t="s">
         <v>40</v>
       </c>
-      <c r="C50" s="33"/>
-      <c r="D50" s="33"/>
-      <c r="E50" s="33" t="s">
+      <c r="C50" s="47"/>
+      <c r="D50" s="47"/>
+      <c r="E50" s="47" t="s">
         <v>31</v>
       </c>
-      <c r="F50" s="33"/>
-      <c r="G50" s="33"/>
+      <c r="F50" s="47"/>
+      <c r="G50" s="47"/>
       <c r="J50">
         <v>50</v>
       </c>
@@ -2075,16 +2075,16 @@
       </c>
     </row>
     <row r="51" spans="2:12" x14ac:dyDescent="0.45">
-      <c r="B51" s="32" t="s">
+      <c r="B51" s="42" t="s">
         <v>26</v>
       </c>
-      <c r="C51" s="32"/>
-      <c r="D51" s="32"/>
-      <c r="E51" s="32" t="s">
+      <c r="C51" s="42"/>
+      <c r="D51" s="42"/>
+      <c r="E51" s="42" t="s">
         <v>32</v>
       </c>
-      <c r="F51" s="32"/>
-      <c r="G51" s="32"/>
+      <c r="F51" s="42"/>
+      <c r="G51" s="42"/>
     </row>
     <row r="52" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B52" s="19"/>
@@ -2103,40 +2103,40 @@
       <c r="G53" s="18"/>
     </row>
     <row r="54" spans="2:12" x14ac:dyDescent="0.45">
-      <c r="B54" s="33" t="s">
+      <c r="B54" s="47" t="s">
         <v>24</v>
       </c>
-      <c r="C54" s="33"/>
-      <c r="D54" s="33"/>
-      <c r="E54" s="33" t="s">
+      <c r="C54" s="47"/>
+      <c r="D54" s="47"/>
+      <c r="E54" s="47" t="s">
         <v>39</v>
       </c>
-      <c r="F54" s="33"/>
-      <c r="G54" s="33"/>
+      <c r="F54" s="47"/>
+      <c r="G54" s="47"/>
       <c r="L54" s="17"/>
     </row>
     <row r="55" spans="2:12" x14ac:dyDescent="0.45">
-      <c r="B55" s="32" t="s">
+      <c r="B55" s="42" t="s">
         <v>20</v>
       </c>
-      <c r="C55" s="32"/>
-      <c r="D55" s="32"/>
-      <c r="E55" s="32" t="s">
+      <c r="C55" s="42"/>
+      <c r="D55" s="42"/>
+      <c r="E55" s="42" t="s">
         <v>33</v>
       </c>
-      <c r="F55" s="32"/>
-      <c r="G55" s="32"/>
+      <c r="F55" s="42"/>
+      <c r="G55" s="42"/>
       <c r="L55" s="17"/>
     </row>
     <row r="56" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B56" s="16"/>
       <c r="C56" s="16"/>
-      <c r="D56" s="31" t="s">
+      <c r="D56" s="43" t="s">
         <v>34</v>
       </c>
-      <c r="E56" s="31"/>
-      <c r="F56" s="31"/>
-      <c r="G56" s="31"/>
+      <c r="E56" s="43"/>
+      <c r="F56" s="43"/>
+      <c r="G56" s="43"/>
       <c r="L56" s="17"/>
     </row>
     <row r="57" spans="2:12" x14ac:dyDescent="0.45">
@@ -2147,12 +2147,62 @@
     </row>
   </sheetData>
   <mergeCells count="78">
-    <mergeCell ref="D1:G1"/>
-    <mergeCell ref="D2:G2"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="E6:G6"/>
-    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="G15:G16"/>
+    <mergeCell ref="C17:G17"/>
+    <mergeCell ref="B54:D54"/>
+    <mergeCell ref="E54:G54"/>
+    <mergeCell ref="D27:G27"/>
+    <mergeCell ref="D28:G28"/>
+    <mergeCell ref="D29:G29"/>
+    <mergeCell ref="D30:G30"/>
+    <mergeCell ref="D31:G31"/>
+    <mergeCell ref="D32:G32"/>
+    <mergeCell ref="D33:G33"/>
+    <mergeCell ref="G24:G25"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="B55:D55"/>
+    <mergeCell ref="E55:G55"/>
+    <mergeCell ref="D34:G34"/>
+    <mergeCell ref="D35:G35"/>
+    <mergeCell ref="D56:G56"/>
+    <mergeCell ref="C38:G38"/>
+    <mergeCell ref="D36:G36"/>
+    <mergeCell ref="C39:G39"/>
+    <mergeCell ref="C40:G40"/>
+    <mergeCell ref="B50:D50"/>
+    <mergeCell ref="E50:G50"/>
+    <mergeCell ref="B51:D51"/>
+    <mergeCell ref="E51:G51"/>
+    <mergeCell ref="C47:G47"/>
+    <mergeCell ref="D22:D23"/>
+    <mergeCell ref="E22:E23"/>
+    <mergeCell ref="F22:F23"/>
+    <mergeCell ref="G22:G23"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="E24:E25"/>
+    <mergeCell ref="F24:F25"/>
+    <mergeCell ref="G20:G21"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="E18:E19"/>
+    <mergeCell ref="F18:F19"/>
+    <mergeCell ref="G18:G19"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="E20:E21"/>
+    <mergeCell ref="F20:F21"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="G13:G14"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="D13:D14"/>
     <mergeCell ref="B15:B16"/>
     <mergeCell ref="C15:C16"/>
     <mergeCell ref="D15:D16"/>
@@ -2169,62 +2219,12 @@
     <mergeCell ref="E9:E10"/>
     <mergeCell ref="F9:F10"/>
     <mergeCell ref="E13:E14"/>
-    <mergeCell ref="F13:F14"/>
-    <mergeCell ref="G13:G14"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="G20:G21"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="D18:D19"/>
-    <mergeCell ref="E18:E19"/>
-    <mergeCell ref="F18:F19"/>
-    <mergeCell ref="G18:G19"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:C21"/>
-    <mergeCell ref="D20:D21"/>
-    <mergeCell ref="E20:E21"/>
-    <mergeCell ref="F20:F21"/>
-    <mergeCell ref="D22:D23"/>
-    <mergeCell ref="E22:E23"/>
-    <mergeCell ref="F22:F23"/>
-    <mergeCell ref="G22:G23"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="E24:E25"/>
-    <mergeCell ref="F24:F25"/>
-    <mergeCell ref="B55:D55"/>
-    <mergeCell ref="E55:G55"/>
-    <mergeCell ref="D34:G34"/>
-    <mergeCell ref="D35:G35"/>
-    <mergeCell ref="D56:G56"/>
-    <mergeCell ref="C38:G38"/>
-    <mergeCell ref="D36:G36"/>
-    <mergeCell ref="C39:G39"/>
-    <mergeCell ref="C40:G40"/>
-    <mergeCell ref="B50:D50"/>
-    <mergeCell ref="E50:G50"/>
-    <mergeCell ref="B51:D51"/>
-    <mergeCell ref="E51:G51"/>
-    <mergeCell ref="C47:G47"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="G15:G16"/>
-    <mergeCell ref="C17:G17"/>
-    <mergeCell ref="B54:D54"/>
-    <mergeCell ref="E54:G54"/>
-    <mergeCell ref="D27:G27"/>
-    <mergeCell ref="D28:G28"/>
-    <mergeCell ref="D29:G29"/>
-    <mergeCell ref="D30:G30"/>
-    <mergeCell ref="D31:G31"/>
-    <mergeCell ref="D32:G32"/>
-    <mergeCell ref="D33:G33"/>
-    <mergeCell ref="G24:G25"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="D1:G1"/>
+    <mergeCell ref="D2:G2"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="E6:G6"/>
+    <mergeCell ref="F4:G4"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
   <pageSetup scale="94" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
fix: soportar 10 materias en templates de 5 semestre (export Excel grupos)
- getGroupTemplateConfig: campo materiaRows (10 para 5°, 9 resto) y abvStartRow +1 (M_5 40, V_5 39)
- buildHorarioGrupoExcelModel: slice limitado por cfg.materiaRows en vez de 9 fijo
- buildHorarioGrupoTemplateCellMap: clearRange parametrizado con materiaRows
- Templates M_5/V_5 actualizados con renglon extra en Materias y Abreviaturas
- Version v1.647
- Artefactos OpenSpec del cambio fix-template-5-semestre-10-materias
</commit_message>
<xml_diff>
--- a/Template_Horarios_Grupos_Matutino_5.xlsx
+++ b/Template_Horarios_Grupos_Matutino_5.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dev\source\repos\CBTis73\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B4604A9-FC43-4B9E-9BAE-E3B067C3E97D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F890FE15-BF25-4D26-A48C-46B5F8DE0FE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="23596" windowHeight="15076" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="GRUPO" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">GRUPO!$A$1:$H$47</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">GRUPO!$A$1:$H$49</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -450,6 +450,96 @@
     <xf numFmtId="0" fontId="11" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="13" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="13" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="10" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="10" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="10" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="13" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="13" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="20" fontId="16" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="16" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="16" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="16" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="11" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="11" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -470,96 +560,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="13" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="13" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="13" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="13" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="11" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="11" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="16" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="16" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="16" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="16" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="10" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="10" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="10" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -637,13 +637,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>148167</xdr:colOff>
-      <xdr:row>49</xdr:row>
+      <xdr:row>51</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>762000</xdr:colOff>
-      <xdr:row>49</xdr:row>
+      <xdr:row>51</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -687,13 +687,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>227541</xdr:colOff>
-      <xdr:row>48</xdr:row>
+      <xdr:row>50</xdr:row>
       <xdr:rowOff>185208</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>854870</xdr:colOff>
-      <xdr:row>48</xdr:row>
+      <xdr:row>50</xdr:row>
       <xdr:rowOff>188119</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -737,13 +737,13 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>83344</xdr:colOff>
-      <xdr:row>52</xdr:row>
+      <xdr:row>54</xdr:row>
       <xdr:rowOff>142875</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>762000</xdr:colOff>
-      <xdr:row>52</xdr:row>
+      <xdr:row>54</xdr:row>
       <xdr:rowOff>154781</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -787,13 +787,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>57151</xdr:colOff>
-      <xdr:row>52</xdr:row>
+      <xdr:row>54</xdr:row>
       <xdr:rowOff>140494</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>819150</xdr:colOff>
-      <xdr:row>52</xdr:row>
+      <xdr:row>54</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
@@ -1137,7 +1137,7 @@
     <tabColor rgb="FFFFC000"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:O58"/>
+  <dimension ref="B1:O60"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="15.1328125" customWidth="1"/>
@@ -1152,22 +1152,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:15" ht="25.5" x14ac:dyDescent="0.75">
-      <c r="D1" s="23" t="s">
+      <c r="D1" s="53" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
+      <c r="E1" s="53"/>
+      <c r="F1" s="53"/>
+      <c r="G1" s="53"/>
       <c r="H1" s="1"/>
       <c r="I1" s="2"/>
     </row>
     <row r="2" spans="2:15" ht="18" x14ac:dyDescent="0.55000000000000004">
-      <c r="D2" s="24" t="s">
+      <c r="D2" s="54" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
+      <c r="E2" s="54"/>
+      <c r="F2" s="54"/>
+      <c r="G2" s="54"/>
       <c r="H2" s="4"/>
       <c r="I2" s="5"/>
       <c r="J2">
@@ -1188,12 +1188,12 @@
     </row>
     <row r="4" spans="2:15" ht="20.65" x14ac:dyDescent="0.6">
       <c r="C4" s="6"/>
-      <c r="D4" s="25"/>
-      <c r="E4" s="25"/>
-      <c r="F4" s="29" t="s">
+      <c r="D4" s="55"/>
+      <c r="E4" s="55"/>
+      <c r="F4" s="59" t="s">
         <v>25</v>
       </c>
-      <c r="G4" s="29"/>
+      <c r="G4" s="59"/>
       <c r="H4" s="6"/>
       <c r="I4" s="5"/>
       <c r="J4">
@@ -1216,15 +1216,15 @@
       <c r="B6" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="26" t="s">
+      <c r="C6" s="56" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="27"/>
-      <c r="E6" s="28" t="s">
+      <c r="D6" s="57"/>
+      <c r="E6" s="58" t="s">
         <v>38</v>
       </c>
-      <c r="F6" s="28"/>
-      <c r="G6" s="28"/>
+      <c r="F6" s="58"/>
+      <c r="G6" s="58"/>
       <c r="H6" s="8"/>
       <c r="I6" s="5"/>
       <c r="J6">
@@ -1281,14 +1281,14 @@
       <c r="O8"/>
     </row>
     <row r="9" spans="2:15" s="13" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B9" s="36" t="s">
+      <c r="B9" s="51" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="34"/>
-      <c r="D9" s="34"/>
-      <c r="E9" s="34"/>
-      <c r="F9" s="34"/>
-      <c r="G9" s="34"/>
+      <c r="C9" s="41"/>
+      <c r="D9" s="41"/>
+      <c r="E9" s="41"/>
+      <c r="F9" s="41"/>
+      <c r="G9" s="41"/>
       <c r="H9" s="12"/>
       <c r="I9" s="5"/>
       <c r="J9">
@@ -1303,12 +1303,12 @@
       <c r="O9"/>
     </row>
     <row r="10" spans="2:15" s="13" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B10" s="37"/>
-      <c r="C10" s="35"/>
-      <c r="D10" s="35"/>
-      <c r="E10" s="35"/>
-      <c r="F10" s="35"/>
-      <c r="G10" s="35"/>
+      <c r="B10" s="52"/>
+      <c r="C10" s="42"/>
+      <c r="D10" s="42"/>
+      <c r="E10" s="42"/>
+      <c r="F10" s="42"/>
+      <c r="G10" s="42"/>
       <c r="H10" s="12"/>
       <c r="I10" s="5"/>
       <c r="J10">
@@ -1323,14 +1323,14 @@
       <c r="O10"/>
     </row>
     <row r="11" spans="2:15" s="13" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B11" s="30" t="s">
+      <c r="B11" s="43" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="34"/>
-      <c r="D11" s="34"/>
-      <c r="E11" s="34"/>
-      <c r="F11" s="34"/>
-      <c r="G11" s="34"/>
+      <c r="C11" s="41"/>
+      <c r="D11" s="41"/>
+      <c r="E11" s="41"/>
+      <c r="F11" s="41"/>
+      <c r="G11" s="41"/>
       <c r="H11" s="12"/>
       <c r="I11" s="5"/>
       <c r="J11">
@@ -1345,12 +1345,12 @@
       <c r="O11"/>
     </row>
     <row r="12" spans="2:15" s="13" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B12" s="31"/>
-      <c r="C12" s="35"/>
-      <c r="D12" s="35"/>
-      <c r="E12" s="35"/>
-      <c r="F12" s="35"/>
-      <c r="G12" s="35"/>
+      <c r="B12" s="44"/>
+      <c r="C12" s="42"/>
+      <c r="D12" s="42"/>
+      <c r="E12" s="42"/>
+      <c r="F12" s="42"/>
+      <c r="G12" s="42"/>
       <c r="H12" s="12"/>
       <c r="I12" s="5"/>
       <c r="J12">
@@ -1365,14 +1365,14 @@
       <c r="O12"/>
     </row>
     <row r="13" spans="2:15" s="13" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B13" s="36" t="s">
+      <c r="B13" s="51" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="34"/>
-      <c r="D13" s="34"/>
-      <c r="E13" s="34"/>
-      <c r="F13" s="34"/>
-      <c r="G13" s="38"/>
+      <c r="C13" s="41"/>
+      <c r="D13" s="41"/>
+      <c r="E13" s="41"/>
+      <c r="F13" s="41"/>
+      <c r="G13" s="49"/>
       <c r="H13" s="12"/>
       <c r="I13" s="5"/>
       <c r="J13">
@@ -1387,12 +1387,12 @@
       <c r="O13"/>
     </row>
     <row r="14" spans="2:15" s="13" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B14" s="37"/>
-      <c r="C14" s="35"/>
-      <c r="D14" s="35"/>
-      <c r="E14" s="35"/>
-      <c r="F14" s="35"/>
-      <c r="G14" s="39"/>
+      <c r="B14" s="52"/>
+      <c r="C14" s="42"/>
+      <c r="D14" s="42"/>
+      <c r="E14" s="42"/>
+      <c r="F14" s="42"/>
+      <c r="G14" s="50"/>
       <c r="H14" s="12"/>
       <c r="I14" s="5"/>
       <c r="J14">
@@ -1407,14 +1407,14 @@
       <c r="O14"/>
     </row>
     <row r="15" spans="2:15" s="13" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B15" s="30" t="s">
+      <c r="B15" s="43" t="s">
         <v>41</v>
       </c>
-      <c r="C15" s="32"/>
-      <c r="D15" s="32"/>
-      <c r="E15" s="32"/>
-      <c r="F15" s="32"/>
-      <c r="G15" s="32"/>
+      <c r="C15" s="26"/>
+      <c r="D15" s="26"/>
+      <c r="E15" s="26"/>
+      <c r="F15" s="26"/>
+      <c r="G15" s="26"/>
       <c r="H15" s="12"/>
       <c r="I15" s="5"/>
       <c r="J15">
@@ -1429,12 +1429,12 @@
       <c r="O15"/>
     </row>
     <row r="16" spans="2:15" s="13" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B16" s="31"/>
-      <c r="C16" s="33"/>
-      <c r="D16" s="33"/>
-      <c r="E16" s="33"/>
-      <c r="F16" s="33"/>
-      <c r="G16" s="33"/>
+      <c r="B16" s="44"/>
+      <c r="C16" s="27"/>
+      <c r="D16" s="27"/>
+      <c r="E16" s="27"/>
+      <c r="F16" s="27"/>
+      <c r="G16" s="27"/>
       <c r="H16" s="12"/>
       <c r="I16" s="5"/>
       <c r="J16">
@@ -1452,13 +1452,13 @@
       <c r="B17" s="22" t="s">
         <v>42</v>
       </c>
-      <c r="C17" s="48" t="s">
+      <c r="C17" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="D17" s="49"/>
-      <c r="E17" s="49"/>
-      <c r="F17" s="49"/>
-      <c r="G17" s="50"/>
+      <c r="D17" s="29"/>
+      <c r="E17" s="29"/>
+      <c r="F17" s="29"/>
+      <c r="G17" s="30"/>
       <c r="H17" s="12"/>
       <c r="I17" s="5"/>
       <c r="J17">
@@ -1473,14 +1473,14 @@
       <c r="O17"/>
     </row>
     <row r="18" spans="2:15" s="13" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B18" s="30" t="s">
+      <c r="B18" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="C18" s="34"/>
-      <c r="D18" s="32"/>
-      <c r="E18" s="34"/>
-      <c r="F18" s="40"/>
-      <c r="G18" s="32"/>
+      <c r="C18" s="41"/>
+      <c r="D18" s="26"/>
+      <c r="E18" s="41"/>
+      <c r="F18" s="47"/>
+      <c r="G18" s="26"/>
       <c r="H18" s="12"/>
       <c r="I18" s="5"/>
       <c r="J18">
@@ -1495,12 +1495,12 @@
       <c r="O18"/>
     </row>
     <row r="19" spans="2:15" s="13" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B19" s="31"/>
-      <c r="C19" s="35"/>
-      <c r="D19" s="33"/>
-      <c r="E19" s="35"/>
-      <c r="F19" s="41"/>
-      <c r="G19" s="33"/>
+      <c r="B19" s="44"/>
+      <c r="C19" s="42"/>
+      <c r="D19" s="27"/>
+      <c r="E19" s="42"/>
+      <c r="F19" s="48"/>
+      <c r="G19" s="27"/>
       <c r="H19" s="12"/>
       <c r="I19" s="5"/>
       <c r="J19">
@@ -1515,14 +1515,14 @@
       <c r="O19"/>
     </row>
     <row r="20" spans="2:15" s="13" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B20" s="30" t="s">
+      <c r="B20" s="43" t="s">
         <v>44</v>
       </c>
-      <c r="C20" s="40"/>
-      <c r="D20" s="32"/>
-      <c r="E20" s="32"/>
-      <c r="F20" s="32"/>
-      <c r="G20" s="32"/>
+      <c r="C20" s="47"/>
+      <c r="D20" s="26"/>
+      <c r="E20" s="26"/>
+      <c r="F20" s="26"/>
+      <c r="G20" s="26"/>
       <c r="H20" s="12"/>
       <c r="I20" s="5"/>
       <c r="J20">
@@ -1537,12 +1537,12 @@
       <c r="O20"/>
     </row>
     <row r="21" spans="2:15" s="13" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B21" s="31"/>
-      <c r="C21" s="41"/>
-      <c r="D21" s="33"/>
-      <c r="E21" s="33"/>
-      <c r="F21" s="33"/>
-      <c r="G21" s="33"/>
+      <c r="B21" s="44"/>
+      <c r="C21" s="48"/>
+      <c r="D21" s="27"/>
+      <c r="E21" s="27"/>
+      <c r="F21" s="27"/>
+      <c r="G21" s="27"/>
       <c r="H21" s="12"/>
       <c r="I21" s="5"/>
       <c r="J21">
@@ -1557,14 +1557,14 @@
       <c r="O21"/>
     </row>
     <row r="22" spans="2:15" s="13" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B22" s="30" t="s">
+      <c r="B22" s="43" t="s">
         <v>13</v>
       </c>
-      <c r="C22" s="32"/>
-      <c r="D22" s="32"/>
-      <c r="E22" s="40"/>
-      <c r="F22" s="40"/>
-      <c r="G22" s="32"/>
+      <c r="C22" s="26"/>
+      <c r="D22" s="26"/>
+      <c r="E22" s="47"/>
+      <c r="F22" s="47"/>
+      <c r="G22" s="26"/>
       <c r="H22" s="12"/>
       <c r="I22" s="5"/>
       <c r="J22">
@@ -1579,12 +1579,12 @@
       <c r="O22"/>
     </row>
     <row r="23" spans="2:15" s="13" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B23" s="31"/>
-      <c r="C23" s="33"/>
-      <c r="D23" s="33"/>
-      <c r="E23" s="41"/>
-      <c r="F23" s="41"/>
-      <c r="G23" s="33"/>
+      <c r="B23" s="44"/>
+      <c r="C23" s="27"/>
+      <c r="D23" s="27"/>
+      <c r="E23" s="48"/>
+      <c r="F23" s="48"/>
+      <c r="G23" s="27"/>
       <c r="H23" s="12"/>
       <c r="I23" s="5"/>
       <c r="J23">
@@ -1599,14 +1599,14 @@
       <c r="O23"/>
     </row>
     <row r="24" spans="2:15" s="13" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B24" s="30" t="s">
+      <c r="B24" s="43" t="s">
         <v>14</v>
       </c>
-      <c r="C24" s="32"/>
-      <c r="D24" s="32"/>
-      <c r="E24" s="32"/>
-      <c r="F24" s="40"/>
-      <c r="G24" s="34"/>
+      <c r="C24" s="26"/>
+      <c r="D24" s="26"/>
+      <c r="E24" s="26"/>
+      <c r="F24" s="47"/>
+      <c r="G24" s="41"/>
       <c r="H24" s="12"/>
       <c r="I24" s="5"/>
       <c r="J24">
@@ -1621,12 +1621,12 @@
       <c r="O24"/>
     </row>
     <row r="25" spans="2:15" s="13" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B25" s="31"/>
-      <c r="C25" s="33"/>
-      <c r="D25" s="33"/>
-      <c r="E25" s="33"/>
-      <c r="F25" s="41"/>
-      <c r="G25" s="35"/>
+      <c r="B25" s="44"/>
+      <c r="C25" s="27"/>
+      <c r="D25" s="27"/>
+      <c r="E25" s="27"/>
+      <c r="F25" s="48"/>
+      <c r="G25" s="42"/>
       <c r="H25" s="12"/>
       <c r="I25" s="5"/>
       <c r="J25">
@@ -1661,12 +1661,12 @@
       <c r="C27" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="D27" s="44" t="s">
+      <c r="D27" s="32" t="s">
         <v>17</v>
       </c>
-      <c r="E27" s="45"/>
-      <c r="F27" s="45"/>
-      <c r="G27" s="46"/>
+      <c r="E27" s="33"/>
+      <c r="F27" s="33"/>
+      <c r="G27" s="34"/>
       <c r="H27" s="12"/>
       <c r="I27" s="5"/>
       <c r="J27">
@@ -1687,10 +1687,10 @@
       <c r="C28" s="15">
         <v>5</v>
       </c>
-      <c r="D28" s="51"/>
-      <c r="E28" s="52"/>
-      <c r="F28" s="52"/>
-      <c r="G28" s="53"/>
+      <c r="D28" s="35"/>
+      <c r="E28" s="36"/>
+      <c r="F28" s="36"/>
+      <c r="G28" s="37"/>
       <c r="H28" s="12"/>
       <c r="I28" s="5"/>
       <c r="J28">
@@ -1711,10 +1711,10 @@
       <c r="C29" s="15">
         <v>5</v>
       </c>
-      <c r="D29" s="51"/>
-      <c r="E29" s="52"/>
-      <c r="F29" s="52"/>
-      <c r="G29" s="53"/>
+      <c r="D29" s="35"/>
+      <c r="E29" s="36"/>
+      <c r="F29" s="36"/>
+      <c r="G29" s="37"/>
       <c r="H29" s="12"/>
       <c r="I29" s="5"/>
       <c r="J29">
@@ -1735,10 +1735,10 @@
       <c r="C30" s="15">
         <v>4</v>
       </c>
-      <c r="D30" s="54"/>
-      <c r="E30" s="55"/>
-      <c r="F30" s="55"/>
-      <c r="G30" s="56"/>
+      <c r="D30" s="38"/>
+      <c r="E30" s="39"/>
+      <c r="F30" s="39"/>
+      <c r="G30" s="40"/>
       <c r="H30" s="12"/>
       <c r="I30" s="5"/>
       <c r="J30">
@@ -1759,10 +1759,10 @@
       <c r="C31" s="15">
         <v>3</v>
       </c>
-      <c r="D31" s="54"/>
-      <c r="E31" s="55"/>
-      <c r="F31" s="55"/>
-      <c r="G31" s="56"/>
+      <c r="D31" s="38"/>
+      <c r="E31" s="39"/>
+      <c r="F31" s="39"/>
+      <c r="G31" s="40"/>
       <c r="H31" s="12"/>
       <c r="I31" s="5"/>
       <c r="J31">
@@ -1779,10 +1779,10 @@
       <c r="C32" s="15">
         <v>1</v>
       </c>
-      <c r="D32" s="51"/>
-      <c r="E32" s="52"/>
-      <c r="F32" s="52"/>
-      <c r="G32" s="53"/>
+      <c r="D32" s="35"/>
+      <c r="E32" s="36"/>
+      <c r="F32" s="36"/>
+      <c r="G32" s="37"/>
       <c r="H32" s="12"/>
       <c r="I32" s="5"/>
       <c r="J32">
@@ -1799,10 +1799,10 @@
       <c r="C33" s="15">
         <v>3</v>
       </c>
-      <c r="D33" s="54"/>
-      <c r="E33" s="55"/>
-      <c r="F33" s="55"/>
-      <c r="G33" s="56"/>
+      <c r="D33" s="38"/>
+      <c r="E33" s="39"/>
+      <c r="F33" s="39"/>
+      <c r="G33" s="40"/>
       <c r="H33" s="12"/>
       <c r="I33" s="5"/>
       <c r="J33">
@@ -1819,10 +1819,10 @@
       <c r="C34" s="15">
         <v>7</v>
       </c>
-      <c r="D34" s="51"/>
-      <c r="E34" s="52"/>
-      <c r="F34" s="52"/>
-      <c r="G34" s="53"/>
+      <c r="D34" s="35"/>
+      <c r="E34" s="36"/>
+      <c r="F34" s="36"/>
+      <c r="G34" s="37"/>
       <c r="H34" s="12"/>
       <c r="I34" s="5"/>
       <c r="J34">
@@ -1839,116 +1839,112 @@
       <c r="C35" s="15">
         <v>5</v>
       </c>
-      <c r="D35" s="51"/>
-      <c r="E35" s="52"/>
-      <c r="F35" s="52"/>
-      <c r="G35" s="53"/>
+      <c r="D35" s="35"/>
+      <c r="E35" s="36"/>
+      <c r="F35" s="36"/>
+      <c r="G35" s="37"/>
       <c r="H35" s="12"/>
       <c r="I35" s="5"/>
     </row>
     <row r="36" spans="2:12" ht="18" x14ac:dyDescent="0.45">
-      <c r="B36" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="C36" s="15">
-        <v>1</v>
-      </c>
-      <c r="D36" s="54"/>
-      <c r="E36" s="55"/>
-      <c r="F36" s="55"/>
-      <c r="G36" s="56"/>
+      <c r="B36" s="15"/>
+      <c r="C36" s="15"/>
+      <c r="D36" s="23"/>
+      <c r="E36" s="24"/>
+      <c r="F36" s="24"/>
+      <c r="G36" s="25"/>
       <c r="H36" s="12"/>
       <c r="I36" s="5"/>
-      <c r="J36">
-        <v>36</v>
-      </c>
-      <c r="L36" s="3" t="s">
-        <v>2</v>
-      </c>
     </row>
     <row r="37" spans="2:12" ht="18" x14ac:dyDescent="0.45">
-      <c r="B37" s="10"/>
-      <c r="C37" s="10"/>
-      <c r="D37" s="10"/>
-      <c r="E37" s="10"/>
-      <c r="F37" s="10"/>
-      <c r="G37" s="10"/>
+      <c r="B37" s="15" t="s">
+        <v>23</v>
+      </c>
+      <c r="C37" s="15">
+        <v>1</v>
+      </c>
+      <c r="D37" s="38"/>
+      <c r="E37" s="39"/>
+      <c r="F37" s="39"/>
+      <c r="G37" s="40"/>
       <c r="H37" s="12"/>
       <c r="I37" s="5"/>
       <c r="J37">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="L37" s="3" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="38" spans="2:12" ht="18" x14ac:dyDescent="0.45">
-      <c r="B38" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="C38" s="44" t="s">
-        <v>19</v>
-      </c>
-      <c r="D38" s="45"/>
-      <c r="E38" s="45"/>
-      <c r="F38" s="45"/>
-      <c r="G38" s="46"/>
+      <c r="B38" s="10"/>
+      <c r="C38" s="10"/>
+      <c r="D38" s="10"/>
+      <c r="E38" s="10"/>
+      <c r="F38" s="10"/>
+      <c r="G38" s="10"/>
+      <c r="H38" s="12"/>
       <c r="I38" s="5"/>
       <c r="J38">
+        <v>37</v>
+      </c>
+      <c r="L38" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39" spans="2:12" ht="18" x14ac:dyDescent="0.45">
+      <c r="B39" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C39" s="32" t="s">
+        <v>19</v>
+      </c>
+      <c r="D39" s="33"/>
+      <c r="E39" s="33"/>
+      <c r="F39" s="33"/>
+      <c r="G39" s="34"/>
+      <c r="I39" s="5"/>
+      <c r="J39">
         <v>39</v>
       </c>
-      <c r="L38" s="3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="39" spans="2:12" ht="18" x14ac:dyDescent="0.45">
-      <c r="B39" s="15"/>
-      <c r="C39" s="51"/>
-      <c r="D39" s="52"/>
-      <c r="E39" s="52"/>
-      <c r="F39" s="52"/>
-      <c r="G39" s="53"/>
-      <c r="I39" s="5"/>
+      <c r="L39" s="3" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="40" spans="2:12" ht="18" x14ac:dyDescent="0.45">
       <c r="B40" s="15"/>
-      <c r="C40" s="51"/>
-      <c r="D40" s="52"/>
-      <c r="E40" s="52"/>
-      <c r="F40" s="52"/>
-      <c r="G40" s="53"/>
+      <c r="C40" s="35"/>
+      <c r="D40" s="36"/>
+      <c r="E40" s="36"/>
+      <c r="F40" s="36"/>
+      <c r="G40" s="37"/>
       <c r="I40" s="5"/>
-      <c r="J40">
-        <v>40</v>
-      </c>
-      <c r="L40" s="3" t="s">
-        <v>2</v>
-      </c>
     </row>
     <row r="41" spans="2:12" ht="18" x14ac:dyDescent="0.45">
       <c r="B41" s="15"/>
-      <c r="C41" s="57"/>
-      <c r="D41" s="58"/>
-      <c r="E41" s="58"/>
-      <c r="F41" s="58"/>
-      <c r="G41" s="59"/>
+      <c r="C41" s="35"/>
+      <c r="D41" s="36"/>
+      <c r="E41" s="36"/>
+      <c r="F41" s="36"/>
+      <c r="G41" s="37"/>
       <c r="I41" s="5"/>
       <c r="J41">
+        <v>40</v>
+      </c>
+      <c r="L41" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="42" spans="2:12" ht="18" x14ac:dyDescent="0.45">
+      <c r="B42" s="15"/>
+      <c r="C42" s="23"/>
+      <c r="D42" s="24"/>
+      <c r="E42" s="24"/>
+      <c r="F42" s="24"/>
+      <c r="G42" s="25"/>
+      <c r="I42" s="5"/>
+      <c r="J42">
         <v>41</v>
-      </c>
-      <c r="L41" s="3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="42" spans="2:12" x14ac:dyDescent="0.45">
-      <c r="B42" s="15"/>
-      <c r="C42" s="57"/>
-      <c r="D42" s="58"/>
-      <c r="E42" s="58"/>
-      <c r="F42" s="58"/>
-      <c r="G42" s="59"/>
-      <c r="J42">
-        <v>42</v>
       </c>
       <c r="L42" s="3" t="s">
         <v>2</v>
@@ -1956,13 +1952,13 @@
     </row>
     <row r="43" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B43" s="15"/>
-      <c r="C43" s="57"/>
-      <c r="D43" s="58"/>
-      <c r="E43" s="58"/>
-      <c r="F43" s="58"/>
-      <c r="G43" s="59"/>
+      <c r="C43" s="23"/>
+      <c r="D43" s="24"/>
+      <c r="E43" s="24"/>
+      <c r="F43" s="24"/>
+      <c r="G43" s="25"/>
       <c r="J43">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="L43" s="3" t="s">
         <v>2</v>
@@ -1970,28 +1966,27 @@
     </row>
     <row r="44" spans="2:12" x14ac:dyDescent="0.45">
       <c r="B44" s="15"/>
-      <c r="C44" s="57"/>
-      <c r="D44" s="58"/>
-      <c r="E44" s="58"/>
-      <c r="F44" s="58"/>
-      <c r="G44" s="59"/>
+      <c r="C44" s="23"/>
+      <c r="D44" s="24"/>
+      <c r="E44" s="24"/>
+      <c r="F44" s="24"/>
+      <c r="G44" s="25"/>
       <c r="J44">
+        <v>43</v>
+      </c>
+      <c r="L44" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="45" spans="2:12" x14ac:dyDescent="0.45">
+      <c r="B45" s="15"/>
+      <c r="C45" s="23"/>
+      <c r="D45" s="24"/>
+      <c r="E45" s="24"/>
+      <c r="F45" s="24"/>
+      <c r="G45" s="25"/>
+      <c r="J45">
         <v>44</v>
-      </c>
-      <c r="L44" s="3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="45" spans="2:12" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="B45" s="15"/>
-      <c r="C45" s="57"/>
-      <c r="D45" s="58"/>
-      <c r="E45" s="58"/>
-      <c r="F45" s="58"/>
-      <c r="G45" s="59"/>
-      <c r="H45" s="9"/>
-      <c r="J45">
-        <v>45</v>
       </c>
       <c r="L45" s="3" t="s">
         <v>2</v>
@@ -1999,14 +1994,14 @@
     </row>
     <row r="46" spans="2:12" ht="15.4" x14ac:dyDescent="0.45">
       <c r="B46" s="15"/>
-      <c r="C46" s="57"/>
-      <c r="D46" s="58"/>
-      <c r="E46" s="58"/>
-      <c r="F46" s="58"/>
-      <c r="G46" s="59"/>
+      <c r="C46" s="23"/>
+      <c r="D46" s="24"/>
+      <c r="E46" s="24"/>
+      <c r="F46" s="24"/>
+      <c r="G46" s="25"/>
       <c r="H46" s="9"/>
       <c r="J46">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="L46" s="3" t="s">
         <v>2</v>
@@ -2014,195 +2009,169 @@
     </row>
     <row r="47" spans="2:12" ht="15.4" x14ac:dyDescent="0.45">
       <c r="B47" s="15"/>
-      <c r="C47" s="51"/>
-      <c r="D47" s="52"/>
-      <c r="E47" s="52"/>
-      <c r="F47" s="52"/>
-      <c r="G47" s="53"/>
+      <c r="C47" s="23"/>
+      <c r="D47" s="24"/>
+      <c r="E47" s="24"/>
+      <c r="F47" s="24"/>
+      <c r="G47" s="25"/>
       <c r="H47" s="9"/>
-      <c r="J47">
-        <v>47</v>
-      </c>
-      <c r="L47" s="3" t="s">
-        <v>2</v>
-      </c>
     </row>
     <row r="48" spans="2:12" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="B48" s="18"/>
-      <c r="C48" s="18"/>
-      <c r="D48" s="18"/>
-      <c r="E48" s="18"/>
-      <c r="F48" s="18"/>
-      <c r="G48" s="18"/>
+      <c r="B48" s="15"/>
+      <c r="C48" s="23"/>
+      <c r="D48" s="24"/>
+      <c r="E48" s="24"/>
+      <c r="F48" s="24"/>
+      <c r="G48" s="25"/>
       <c r="H48" s="9"/>
       <c r="J48">
+        <v>46</v>
+      </c>
+      <c r="L48" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="49" spans="2:12" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="B49" s="15"/>
+      <c r="C49" s="35"/>
+      <c r="D49" s="36"/>
+      <c r="E49" s="36"/>
+      <c r="F49" s="36"/>
+      <c r="G49" s="37"/>
+      <c r="H49" s="9"/>
+      <c r="J49">
+        <v>47</v>
+      </c>
+      <c r="L49" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="50" spans="2:12" ht="15.4" x14ac:dyDescent="0.45">
+      <c r="B50" s="18"/>
+      <c r="C50" s="18"/>
+      <c r="D50" s="18"/>
+      <c r="E50" s="18"/>
+      <c r="F50" s="18"/>
+      <c r="G50" s="18"/>
+      <c r="H50" s="9"/>
+      <c r="J50">
         <v>48</v>
       </c>
-      <c r="L48" s="3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="49" spans="2:12" x14ac:dyDescent="0.45">
-      <c r="B49" s="18"/>
-      <c r="C49" s="18"/>
-      <c r="D49" s="18"/>
-      <c r="E49" s="18"/>
-      <c r="F49" s="18"/>
-      <c r="G49" s="18"/>
-      <c r="J49">
+      <c r="L50" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="51" spans="2:12" x14ac:dyDescent="0.45">
+      <c r="B51" s="18"/>
+      <c r="C51" s="18"/>
+      <c r="D51" s="18"/>
+      <c r="E51" s="18"/>
+      <c r="F51" s="18"/>
+      <c r="G51" s="18"/>
+      <c r="J51">
         <v>49</v>
       </c>
-      <c r="L49" s="3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="50" spans="2:12" x14ac:dyDescent="0.45">
-      <c r="B50" s="47" t="s">
+      <c r="L51" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="52" spans="2:12" x14ac:dyDescent="0.45">
+      <c r="B52" s="31" t="s">
         <v>40</v>
       </c>
-      <c r="C50" s="47"/>
-      <c r="D50" s="47"/>
-      <c r="E50" s="47" t="s">
+      <c r="C52" s="31"/>
+      <c r="D52" s="31"/>
+      <c r="E52" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="F50" s="47"/>
-      <c r="G50" s="47"/>
-      <c r="J50">
+      <c r="F52" s="31"/>
+      <c r="G52" s="31"/>
+      <c r="J52">
         <v>50</v>
       </c>
-      <c r="L50" s="3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="51" spans="2:12" x14ac:dyDescent="0.45">
-      <c r="B51" s="42" t="s">
+      <c r="L52" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="53" spans="2:12" x14ac:dyDescent="0.45">
+      <c r="B53" s="45" t="s">
         <v>26</v>
       </c>
-      <c r="C51" s="42"/>
-      <c r="D51" s="42"/>
-      <c r="E51" s="42" t="s">
+      <c r="C53" s="45"/>
+      <c r="D53" s="45"/>
+      <c r="E53" s="45" t="s">
         <v>32</v>
       </c>
-      <c r="F51" s="42"/>
-      <c r="G51" s="42"/>
-    </row>
-    <row r="52" spans="2:12" x14ac:dyDescent="0.45">
-      <c r="B52" s="19"/>
-      <c r="C52" s="19"/>
-      <c r="D52" s="19"/>
-      <c r="E52" s="19"/>
-      <c r="F52" s="19"/>
-      <c r="G52" s="19"/>
-    </row>
-    <row r="53" spans="2:12" x14ac:dyDescent="0.45">
-      <c r="B53" s="18"/>
-      <c r="C53" s="18"/>
-      <c r="D53" s="18"/>
-      <c r="E53" s="18"/>
-      <c r="F53" s="18"/>
-      <c r="G53" s="18"/>
+      <c r="F53" s="45"/>
+      <c r="G53" s="45"/>
     </row>
     <row r="54" spans="2:12" x14ac:dyDescent="0.45">
-      <c r="B54" s="47" t="s">
+      <c r="B54" s="19"/>
+      <c r="C54" s="19"/>
+      <c r="D54" s="19"/>
+      <c r="E54" s="19"/>
+      <c r="F54" s="19"/>
+      <c r="G54" s="19"/>
+    </row>
+    <row r="55" spans="2:12" x14ac:dyDescent="0.45">
+      <c r="B55" s="18"/>
+      <c r="C55" s="18"/>
+      <c r="D55" s="18"/>
+      <c r="E55" s="18"/>
+      <c r="F55" s="18"/>
+      <c r="G55" s="18"/>
+    </row>
+    <row r="56" spans="2:12" x14ac:dyDescent="0.45">
+      <c r="B56" s="31" t="s">
         <v>24</v>
       </c>
-      <c r="C54" s="47"/>
-      <c r="D54" s="47"/>
-      <c r="E54" s="47" t="s">
+      <c r="C56" s="31"/>
+      <c r="D56" s="31"/>
+      <c r="E56" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="F54" s="47"/>
-      <c r="G54" s="47"/>
-      <c r="L54" s="17"/>
-    </row>
-    <row r="55" spans="2:12" x14ac:dyDescent="0.45">
-      <c r="B55" s="42" t="s">
+      <c r="F56" s="31"/>
+      <c r="G56" s="31"/>
+      <c r="L56" s="17"/>
+    </row>
+    <row r="57" spans="2:12" x14ac:dyDescent="0.45">
+      <c r="B57" s="45" t="s">
         <v>20</v>
       </c>
-      <c r="C55" s="42"/>
-      <c r="D55" s="42"/>
-      <c r="E55" s="42" t="s">
+      <c r="C57" s="45"/>
+      <c r="D57" s="45"/>
+      <c r="E57" s="45" t="s">
         <v>33</v>
       </c>
-      <c r="F55" s="42"/>
-      <c r="G55" s="42"/>
-      <c r="L55" s="17"/>
-    </row>
-    <row r="56" spans="2:12" x14ac:dyDescent="0.45">
-      <c r="B56" s="16"/>
-      <c r="C56" s="16"/>
-      <c r="D56" s="43" t="s">
+      <c r="F57" s="45"/>
+      <c r="G57" s="45"/>
+      <c r="L57" s="17"/>
+    </row>
+    <row r="58" spans="2:12" x14ac:dyDescent="0.45">
+      <c r="B58" s="16"/>
+      <c r="C58" s="16"/>
+      <c r="D58" s="46" t="s">
         <v>34</v>
       </c>
-      <c r="E56" s="43"/>
-      <c r="F56" s="43"/>
-      <c r="G56" s="43"/>
-      <c r="L56" s="17"/>
-    </row>
-    <row r="57" spans="2:12" x14ac:dyDescent="0.45">
-      <c r="L57" s="17"/>
-    </row>
-    <row r="58" spans="2:12" x14ac:dyDescent="0.45">
+      <c r="E58" s="46"/>
+      <c r="F58" s="46"/>
+      <c r="G58" s="46"/>
       <c r="L58" s="17"/>
+    </row>
+    <row r="59" spans="2:12" x14ac:dyDescent="0.45">
+      <c r="L59" s="17"/>
+    </row>
+    <row r="60" spans="2:12" x14ac:dyDescent="0.45">
+      <c r="L60" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="78">
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="G15:G16"/>
-    <mergeCell ref="C17:G17"/>
-    <mergeCell ref="B54:D54"/>
-    <mergeCell ref="E54:G54"/>
-    <mergeCell ref="D27:G27"/>
-    <mergeCell ref="D28:G28"/>
-    <mergeCell ref="D29:G29"/>
-    <mergeCell ref="D30:G30"/>
-    <mergeCell ref="D31:G31"/>
-    <mergeCell ref="D32:G32"/>
-    <mergeCell ref="D33:G33"/>
-    <mergeCell ref="G24:G25"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="B55:D55"/>
-    <mergeCell ref="E55:G55"/>
-    <mergeCell ref="D34:G34"/>
-    <mergeCell ref="D35:G35"/>
-    <mergeCell ref="D56:G56"/>
-    <mergeCell ref="C38:G38"/>
-    <mergeCell ref="D36:G36"/>
-    <mergeCell ref="C39:G39"/>
-    <mergeCell ref="C40:G40"/>
-    <mergeCell ref="B50:D50"/>
-    <mergeCell ref="E50:G50"/>
-    <mergeCell ref="B51:D51"/>
-    <mergeCell ref="E51:G51"/>
-    <mergeCell ref="C47:G47"/>
-    <mergeCell ref="D22:D23"/>
-    <mergeCell ref="E22:E23"/>
-    <mergeCell ref="F22:F23"/>
-    <mergeCell ref="G22:G23"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="D24:D25"/>
-    <mergeCell ref="E24:E25"/>
-    <mergeCell ref="F24:F25"/>
-    <mergeCell ref="G20:G21"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="D18:D19"/>
-    <mergeCell ref="E18:E19"/>
-    <mergeCell ref="F18:F19"/>
-    <mergeCell ref="G18:G19"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="C20:C21"/>
-    <mergeCell ref="D20:D21"/>
-    <mergeCell ref="E20:E21"/>
-    <mergeCell ref="F20:F21"/>
-    <mergeCell ref="F13:F14"/>
-    <mergeCell ref="G13:G14"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="D1:G1"/>
+    <mergeCell ref="D2:G2"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="E6:G6"/>
+    <mergeCell ref="F4:G4"/>
     <mergeCell ref="B15:B16"/>
     <mergeCell ref="C15:C16"/>
     <mergeCell ref="D15:D16"/>
@@ -2219,12 +2188,62 @@
     <mergeCell ref="E9:E10"/>
     <mergeCell ref="F9:F10"/>
     <mergeCell ref="E13:E14"/>
-    <mergeCell ref="D1:G1"/>
-    <mergeCell ref="D2:G2"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="E6:G6"/>
-    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="F13:F14"/>
+    <mergeCell ref="G13:G14"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="G20:G21"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="E18:E19"/>
+    <mergeCell ref="F18:F19"/>
+    <mergeCell ref="G18:G19"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="E20:E21"/>
+    <mergeCell ref="F20:F21"/>
+    <mergeCell ref="D22:D23"/>
+    <mergeCell ref="E22:E23"/>
+    <mergeCell ref="F22:F23"/>
+    <mergeCell ref="G22:G23"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="D24:D25"/>
+    <mergeCell ref="E24:E25"/>
+    <mergeCell ref="F24:F25"/>
+    <mergeCell ref="B57:D57"/>
+    <mergeCell ref="E57:G57"/>
+    <mergeCell ref="D34:G34"/>
+    <mergeCell ref="D35:G35"/>
+    <mergeCell ref="D58:G58"/>
+    <mergeCell ref="C39:G39"/>
+    <mergeCell ref="D37:G37"/>
+    <mergeCell ref="C40:G40"/>
+    <mergeCell ref="C41:G41"/>
+    <mergeCell ref="B52:D52"/>
+    <mergeCell ref="E52:G52"/>
+    <mergeCell ref="B53:D53"/>
+    <mergeCell ref="E53:G53"/>
+    <mergeCell ref="C49:G49"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="G15:G16"/>
+    <mergeCell ref="C17:G17"/>
+    <mergeCell ref="B56:D56"/>
+    <mergeCell ref="E56:G56"/>
+    <mergeCell ref="D27:G27"/>
+    <mergeCell ref="D28:G28"/>
+    <mergeCell ref="D29:G29"/>
+    <mergeCell ref="D30:G30"/>
+    <mergeCell ref="D31:G31"/>
+    <mergeCell ref="D32:G32"/>
+    <mergeCell ref="D33:G33"/>
+    <mergeCell ref="G24:G25"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="C22:C23"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
   <pageSetup scale="94" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>